<commit_message>
Publish category-aligned workforce dashboard
</commit_message>
<xml_diff>
--- a/Aditi_Workforce_Dashboard_Upload_Template.xlsx
+++ b/Aditi_Workforce_Dashboard_Upload_Template.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R61d39ccd744d4bc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity" sheetId="2" r:id="Rfb84c1677032425d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contractors" sheetId="3" r:id="R0ddc0a72d8e74245"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrition" sheetId="4" r:id="Ra4e37db8737541ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrition BU Detail" sheetId="5" r:id="R1664f938b6074bee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ODC Breakdown" sheetId="6" r:id="Ra5cf73ecb04849af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R4d9d5a4efce24a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exit Interview" sheetId="8" r:id="R065402dfd6b64749"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rac9d5d1d5b144d7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity" sheetId="2" r:id="Re085e0aa1e254b0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contractors" sheetId="3" r:id="Raf6eed66b1764d81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Deployment" sheetId="4" r:id="R82b13afdd7bc4384"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrition" sheetId="5" r:id="R7a7df272973e473f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrition BU Detail" sheetId="6" r:id="Rb595612cc8b34f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ODC Breakdown" sheetId="7" r:id="Rda9b1099418849e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="8" r:id="Rcb679cea28cb4559"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exit Interview" sheetId="9" r:id="Rae0b7caf2a724122"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -80,7 +81,13 @@
     </x:fill>
   </x:fills>
   <x:borders count="2">
-    <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFDDE6EB"/>
@@ -94,6 +101,7 @@
       <x:bottom style="thin">
         <x:color rgb="FFDDE6EB"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
@@ -364,7 +372,7 @@
         <x:v>ONE-GO UPDATE</x:v>
       </x:c>
       <x:c r="B4" s="8" t="str">
-        <x:v>Capacity, contractors, consolidated attrition, ODC bifurcation, settings and confidential exit-interview content are imported together.</x:v>
+        <x:v>Capacity, India ToD contractors, combined client deployment, both attrition views, ODC bifurcation, settings and confidential exit-interview content are imported together.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -385,10 +393,10 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="5" t="str">
-        <x:v>ROW NAMES</x:v>
+        <x:v>CATEGORY RULES</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
-        <x:v>Keep the supplied business-unit and ODC category names unchanged so the dashboard can map them correctly.</x:v>
+        <x:v>Use the source Category policy: Internal Employee and Internal Billable count in overall attrition; Track Separate and Fixed Term Contractors remain separate; Not To Count In Attrition is excluded.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -669,9 +677,7 @@
       <x:c r="G6" s="16" t="str">
         <x:v>9 × Billable fixed-term contractor positions</x:v>
       </x:c>
-      <x:c r="H6" s="16" t="str">
-        <x:v>Name not provided</x:v>
-      </x:c>
+      <x:c r="H6" s="16" t="str"/>
       <x:c r="I6" s="16" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1014,6 +1020,343 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="17" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="B1" s="17" t="str">
+        <x:v>India ToD HC</x:v>
+      </x:c>
+      <x:c r="C1" s="17" t="str">
+        <x:v>ODC HC</x:v>
+      </x:c>
+      <x:c r="D1" s="17" t="str">
+        <x:v>Combined HC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="16" t="str">
+        <x:v>Standard Chartered</x:v>
+      </x:c>
+      <x:c r="B2" s="16" t="n">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="C2" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D2" s="16" t="n">
+        <x:v>156</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="16" t="str">
+        <x:v>Amazon</x:v>
+      </x:c>
+      <x:c r="B3" s="16" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="C3" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D3" s="16" t="n">
+        <x:v>71</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>PayPal</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="n">
+        <x:v>64</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="16" t="str">
+        <x:v>T-Mobile</x:v>
+      </x:c>
+      <x:c r="B5" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C5" s="16" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D5" s="16" t="n">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="16" t="str">
+        <x:v>Wabtec</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C6" s="16" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="D6" s="16" t="n">
+        <x:v>39</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="16" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="C7" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D7" s="16" t="n">
+        <x:v>30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="16" t="str">
+        <x:v>Caterpillar</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C8" s="16" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D8" s="16" t="n">
+        <x:v>27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="16" t="str">
+        <x:v>MasterCard</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C9" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="16" t="n">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="16" t="str">
+        <x:v>LinkedIn</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C10" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="16" t="n">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="16" t="str">
+        <x:v>Rubrik</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C11" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D11" s="16" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="16" t="str">
+        <x:v>AI Labs</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C12" s="16" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D12" s="16" t="n">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="16" t="str">
+        <x:v>Salesforce</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C13" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D13" s="16" t="n">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="16" t="str">
+        <x:v>Diageo PLC</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C14" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="16" t="str">
+        <x:v>Q2 Financials</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C15" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D15" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="16" t="str">
+        <x:v>Bench</x:v>
+      </x:c>
+      <x:c r="B16" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C16" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D16" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="16" t="str">
+        <x:v>PepsiCo</x:v>
+      </x:c>
+      <x:c r="B17" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C17" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D17" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="16" t="str">
+        <x:v>GE Aerospace</x:v>
+      </x:c>
+      <x:c r="B18" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C18" s="16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D18" s="16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="16" t="str">
+        <x:v>Overhead</x:v>
+      </x:c>
+      <x:c r="B19" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C19" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D19" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="16" t="str">
+        <x:v>Intuit</x:v>
+      </x:c>
+      <x:c r="B20" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C20" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D20" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="16" t="str">
+        <x:v>Sales</x:v>
+      </x:c>
+      <x:c r="B21" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C21" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="16" t="str">
+        <x:v>Practice</x:v>
+      </x:c>
+      <x:c r="B22" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C22" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D22" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="16" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="B23" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C23" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D23" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="8" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="8" hidden="0" customWidth="1"/>
@@ -1118,16 +1461,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E3" s="16" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F3" s="16" t="n">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="G3" s="18" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0.191489</x:v>
       </x:c>
       <x:c r="H3" s="18" t="n">
-        <x:v>0.24</x:v>
+        <x:v>0.229787</x:v>
       </x:c>
       <x:c r="I3" s="16" t="n">
         <x:v>139</x:v>
@@ -1147,25 +1490,25 @@
         <x:v>ODC Internal</x:v>
       </x:c>
       <x:c r="B4" s="16" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C4" s="16" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D4" s="16" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="16" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F4" s="16" t="n">
-        <x:v>14</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G4" s="18" t="n">
-        <x:v>1.04</x:v>
+        <x:v>0.148148</x:v>
       </x:c>
       <x:c r="H4" s="18" t="n">
-        <x:v>1.24</x:v>
+        <x:v>0.177778</x:v>
       </x:c>
       <x:c r="I4" s="16" t="n">
         <x:v>12</x:v>
@@ -1185,25 +1528,25 @@
         <x:v>ODC Internal Billable</x:v>
       </x:c>
       <x:c r="B5" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C5" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D5" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E5" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F5" s="16" t="n">
-        <x:v>1</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G5" s="18" t="n">
-        <x:v>0.01</x:v>
+        <x:v>0.127907</x:v>
       </x:c>
       <x:c r="H5" s="18" t="n">
-        <x:v>0.01</x:v>
+        <x:v>0.153488</x:v>
       </x:c>
       <x:c r="I5" s="16" t="n">
         <x:v>93</x:v>
@@ -1226,7 +1569,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C6" s="16" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D6" s="16" t="n">
         <x:v>8</x:v>
@@ -1235,13 +1578,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="16" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G6" s="18" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.430769</x:v>
       </x:c>
       <x:c r="H6" s="18" t="n">
-        <x:v>0.48</x:v>
+        <x:v>0.516923</x:v>
       </x:c>
       <x:c r="I6" s="16" t="n">
         <x:v>34</x:v>
@@ -1253,7 +1596,7 @@
         <x:v>32.5</x:v>
       </x:c>
       <x:c r="L6" s="16" t="str">
-        <x:v>No</x:v>
+        <x:v>No – track separately</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1308,16 +1651,16 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="E8" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F8" s="16" t="n">
-        <x:v>161</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="G8" s="18" t="n">
-        <x:v>0.51</x:v>
+        <x:v>0.515008</x:v>
       </x:c>
       <x:c r="H8" s="18" t="n">
-        <x:v>0.61</x:v>
+        <x:v>0.618009</x:v>
       </x:c>
       <x:c r="I8" s="16" t="n">
         <x:v>259</x:v>
@@ -1329,7 +1672,7 @@
         <x:v>316.5</x:v>
       </x:c>
       <x:c r="L8" s="16" t="str">
-        <x:v>No</x:v>
+        <x:v>No – track separately</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1337,7 +1680,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1356,7 +1699,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="17" t="str">
-        <x:v>BU</x:v>
+        <x:v>Business Unit</x:v>
       </x:c>
       <x:c r="B1" s="17" t="str">
         <x:v>Q1</x:v>
@@ -1391,7 +1734,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="16" t="str">
-        <x:v>US recruited (TOD &amp; DES)</x:v>
+        <x:v>US Recruitment</x:v>
       </x:c>
       <x:c r="B2" s="16" t="n">
         <x:v>14</x:v>
@@ -1402,7 +1745,9 @@
       <x:c r="D2" s="16" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E2" s="16" t="str"/>
+      <x:c r="E2" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F2" s="16" t="n">
         <x:v>34</x:v>
       </x:c>
@@ -1424,7 +1769,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="16" t="str">
-        <x:v>India Recruitment (TOD &amp; DES)</x:v>
+        <x:v>India Recruitment</x:v>
       </x:c>
       <x:c r="B3" s="16" t="n">
         <x:v>7</x:v>
@@ -1435,15 +1780,17 @@
       <x:c r="D3" s="16" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E3" s="16" t="str"/>
+      <x:c r="E3" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F3" s="16" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="G3" s="18" t="n">
-        <x:v>0.44</x:v>
+        <x:v>0.441176</x:v>
       </x:c>
       <x:c r="H3" s="18" t="n">
-        <x:v>0.53</x:v>
+        <x:v>0.529412</x:v>
       </x:c>
       <x:c r="I3" s="16" t="n">
         <x:v>36</x:v>
@@ -1468,15 +1815,17 @@
       <x:c r="D4" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E4" s="16" t="str"/>
+      <x:c r="E4" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F4" s="16" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="G4" s="18" t="n">
-        <x:v>0.36</x:v>
+        <x:v>0.358974</x:v>
       </x:c>
       <x:c r="H4" s="18" t="n">
-        <x:v>0.43</x:v>
+        <x:v>0.430769</x:v>
       </x:c>
       <x:c r="I4" s="16" t="n">
         <x:v>21</x:v>
@@ -1501,15 +1850,17 @@
       <x:c r="D5" s="16" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E5" s="16" t="str"/>
+      <x:c r="E5" s="16" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F5" s="16" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="G5" s="18" t="n">
-        <x:v>0.23</x:v>
+        <x:v>0.232258</x:v>
       </x:c>
       <x:c r="H5" s="18" t="n">
-        <x:v>0.28</x:v>
+        <x:v>0.27871</x:v>
       </x:c>
       <x:c r="I5" s="16" t="n">
         <x:v>79</x:v>
@@ -1523,204 +1874,37 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="16" t="str">
-        <x:v>India ToD Contractors</x:v>
+        <x:v>ODC</x:v>
       </x:c>
       <x:c r="B6" s="16" t="n">
-        <x:v>66</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C6" s="16" t="n">
-        <x:v>37</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D6" s="16" t="n">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="E6" s="16" t="str"/>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E6" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="F6" s="16" t="n">
-        <x:v>161</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="G6" s="18" t="n">
-        <x:v>0.51</x:v>
+        <x:v>0.191489</x:v>
       </x:c>
       <x:c r="H6" s="18" t="n">
-        <x:v>0.61</x:v>
+        <x:v>0.229787</x:v>
       </x:c>
       <x:c r="I6" s="16" t="n">
-        <x:v>259</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="J6" s="16" t="n">
-        <x:v>370</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="K6" s="16" t="n">
-        <x:v>314.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="16" t="str">
-        <x:v>ODC</x:v>
-      </x:c>
-      <x:c r="B7" s="16" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C7" s="16" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D7" s="16" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E7" s="16" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F7" s="16" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="G7" s="18" t="n">
-        <x:v>0.2</x:v>
-      </x:c>
-      <x:c r="H7" s="18" t="n">
-        <x:v>0.24</x:v>
-      </x:c>
-      <x:c r="I7" s="16" t="n">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="J7" s="16" t="n">
-        <x:v>143</x:v>
-      </x:c>
-      <x:c r="K7" s="16" t="n">
         <x:v>141</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="16" t="str">
-        <x:v>ODC Internal</x:v>
-      </x:c>
-      <x:c r="B8" s="16" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C8" s="16" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="D8" s="16" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E8" s="16" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F8" s="16" t="str"/>
-      <x:c r="G8" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H8" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I8" s="16" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="J8" s="16" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="K8" s="16" t="n">
-        <x:v>13.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="16" t="str">
-        <x:v>ODC Billable</x:v>
-      </x:c>
-      <x:c r="B9" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C9" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D9" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E9" s="16" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F9" s="16" t="str"/>
-      <x:c r="G9" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H9" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I9" s="16" t="n">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="J9" s="16" t="n">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="K9" s="16" t="n">
-        <x:v>86</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="16" t="str">
-        <x:v>ODC Fixed Term Contractors</x:v>
-      </x:c>
-      <x:c r="B10" s="16" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C10" s="16" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D10" s="16" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E10" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F10" s="16" t="str"/>
-      <x:c r="G10" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H10" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I10" s="16" t="n">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="J10" s="16" t="n">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="K10" s="16" t="n">
-        <x:v>32.5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>Total</x:v>
-      </x:c>
-      <x:c r="B11" s="16" t="n">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="C11" s="16" t="n">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="D11" s="16" t="n">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="E11" s="16" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="F11" s="16" t="n">
-        <x:v>263</x:v>
-      </x:c>
-      <x:c r="G11" s="18" t="n">
-        <x:v>0.33</x:v>
-      </x:c>
-      <x:c r="H11" s="18" t="n">
-        <x:v>0.4</x:v>
-      </x:c>
-      <x:c r="I11" s="16" t="n">
-        <x:v>752</x:v>
-      </x:c>
-      <x:c r="J11" s="16" t="n">
-        <x:v>821</x:v>
-      </x:c>
-      <x:c r="K11" s="16" t="n">
-        <x:v>786.5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1728,7 +1912,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1789,7 +1973,7 @@
         <x:v>Shared Internal</x:v>
       </x:c>
       <x:c r="B7" s="16" t="n">
-        <x:v>184</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1797,7 +1981,7 @@
         <x:v>Shared Interns</x:v>
       </x:c>
       <x:c r="B8" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1805,7 +1989,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1826,7 +2010,7 @@
         <x:v>Snapshot Date</x:v>
       </x:c>
       <x:c r="B2" s="16" t="str">
-        <x:v>13 Oct 2026</x:v>
+        <x:v>14 Oct 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1834,7 +2018,7 @@
         <x:v>Overall Internal Attrition</x:v>
       </x:c>
       <x:c r="B3" s="18" t="n">
-        <x:v>0.36</x:v>
+        <x:v>0.35</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1866,7 +2050,7 @@
         <x:v>Exit Callout</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
-        <x:v>Positive culture and resources; managerial conduct requires review</x:v>
+        <x:v>No exit-interview data supplied in the current workbook</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1874,7 +2058,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1895,26 +2079,9 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="16" t="str">
-        <x:v>Positive</x:v>
-      </x:c>
-      <x:c r="B2" s="16" t="str">
-        <x:v>Enter positive theme</x:v>
-      </x:c>
-      <x:c r="C2" s="16" t="str">
-        <x:v>Enter anonymised details for authorised leadership use.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="16" t="str">
-        <x:v>Concern</x:v>
-      </x:c>
-      <x:c r="B3" s="16" t="str">
-        <x:v>Enter concern theme</x:v>
-      </x:c>
-      <x:c r="C3" s="16" t="str">
-        <x:v>Do not enter employee names; summarise confidential feedback.</x:v>
-      </x:c>
+      <x:c r="A2" s="16" t="str"/>
+      <x:c r="B2" s="16" t="str"/>
+      <x:c r="C2" s="16" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Publish simplified dashboard and corrected attrition rules
</commit_message>
<xml_diff>
--- a/Aditi_Workforce_Dashboard_Upload_Template.xlsx
+++ b/Aditi_Workforce_Dashboard_Upload_Template.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rac9d5d1d5b144d7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity" sheetId="2" r:id="Re085e0aa1e254b0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contractors" sheetId="3" r:id="Raf6eed66b1764d81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Deployment" sheetId="4" r:id="R82b13afdd7bc4384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrition" sheetId="5" r:id="R7a7df272973e473f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrition BU Detail" sheetId="6" r:id="Rb595612cc8b34f29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ODC Breakdown" sheetId="7" r:id="Rda9b1099418849e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="8" r:id="Rcb679cea28cb4559"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exit Interview" sheetId="9" r:id="Rae0b7caf2a724122"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rffb1a378b8e34e76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity" sheetId="2" r:id="R93316a08e2054dec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contractors" sheetId="3" r:id="Rf797b2c7b2a94457"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Deployment" sheetId="4" r:id="R671ed1338b474be0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrition" sheetId="5" r:id="R414976d6997c49e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrition BU Detail" sheetId="6" r:id="Rbc4c83fe69714d82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ODC Breakdown" sheetId="7" r:id="Rc4dac11e95ad4e5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="India ToD Exit Clients" sheetId="8" r:id="Rb6ea08da2d3047b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="9" r:id="R259ecaf3856642b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exit Interview" sheetId="10" r:id="Raffcc8b2009644b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -396,7 +397,7 @@
         <x:v>CATEGORY RULES</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
-        <x:v>Use the source Category policy: Internal Employee and Internal Billable count in overall attrition; Track Separate and Fixed Term Contractors remain separate; Not To Count In Attrition is excluded.</x:v>
+        <x:v>Overall attrition includes Recruitment &amp; Client Services, Business Operations and ODC Internal only. Exclude ODC Internal Billable, ODC Fixed Term Contractors, India ToD Contractors and Not To Count In Attrition.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -419,6 +420,36 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="38" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="17" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="B1" s="17" t="str">
+        <x:v>Observation</x:v>
+      </x:c>
+      <x:c r="C1" s="17" t="str">
+        <x:v>Details</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="16" t="str"/>
+      <x:c r="B2" s="16" t="str"/>
+      <x:c r="C2" s="16" t="str"/>
+    </x:row>
+  </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -441,9 +472,6 @@
     <x:col min="12" max="12" width="27" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="8" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="10" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="10" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="10" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -489,15 +517,6 @@
       <x:c r="N1" s="17" t="str">
         <x:v>PIP People</x:v>
       </x:c>
-      <x:c r="O1" s="17" t="str">
-        <x:v>Closed</x:v>
-      </x:c>
-      <x:c r="P1" s="17" t="str">
-        <x:v>On Hold</x:v>
-      </x:c>
-      <x:c r="Q1" s="17" t="str">
-        <x:v>Cancelled</x:v>
-      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="16" t="str">
@@ -534,9 +553,6 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="N2" s="16" t="str"/>
-      <x:c r="O2" s="16" t="str"/>
-      <x:c r="P2" s="16" t="str"/>
-      <x:c r="Q2" s="16" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="16" t="str">
@@ -573,9 +589,6 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N3" s="16" t="str"/>
-      <x:c r="O3" s="16" t="str"/>
-      <x:c r="P3" s="16" t="str"/>
-      <x:c r="Q3" s="16" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="16" t="str">
@@ -612,9 +625,6 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N4" s="16" t="str"/>
-      <x:c r="O4" s="16" t="str"/>
-      <x:c r="P4" s="16" t="str"/>
-      <x:c r="Q4" s="16" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="str">
@@ -651,13 +661,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N5" s="16" t="str"/>
-      <x:c r="O5" s="16" t="str"/>
-      <x:c r="P5" s="16" t="str"/>
-      <x:c r="Q5" s="16" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="16" t="str">
-        <x:v>ODC / DES</x:v>
+        <x:v>ODC</x:v>
       </x:c>
       <x:c r="B6" s="16" t="n">
         <x:v>152</x:v>
@@ -690,9 +697,6 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="N6" s="16" t="str"/>
-      <x:c r="O6" s="16" t="str"/>
-      <x:c r="P6" s="16" t="str"/>
-      <x:c r="Q6" s="16" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1558,7 +1562,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="L5" s="16" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No – excluded</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1968,28 +1972,137 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="16" t="str">
-        <x:v>Shared Internal</x:v>
-      </x:c>
-      <x:c r="B7" s="16" t="n">
-        <x:v>182</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="16" t="str">
-        <x:v>Shared Interns</x:v>
-      </x:c>
-      <x:c r="B8" s="16" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="17" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="B1" s="17" t="str">
+        <x:v>Exits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="16" t="str">
+        <x:v>PayPal</x:v>
+      </x:c>
+      <x:c r="B2" s="16" t="n">
+        <x:v>55</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="16" t="str">
+        <x:v>Amazon</x:v>
+      </x:c>
+      <x:c r="B3" s="16" t="n">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Standard Chartered</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="n">
+        <x:v>27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="16" t="str">
+        <x:v>Microsoft</x:v>
+      </x:c>
+      <x:c r="B5" s="16" t="n">
+        <x:v>23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="16" t="str">
+        <x:v>LinkedIn</x:v>
+      </x:c>
+      <x:c r="B6" s="16" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="16" t="str">
+        <x:v>MasterCard</x:v>
+      </x:c>
+      <x:c r="B7" s="16" t="n">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="16" t="str">
+        <x:v>Diageo PLC</x:v>
+      </x:c>
+      <x:c r="B8" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="16" t="str">
+        <x:v>Salesforce</x:v>
+      </x:c>
+      <x:c r="B9" s="16" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="16" t="str">
+        <x:v>Q2 Financials</x:v>
+      </x:c>
+      <x:c r="B10" s="16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="16" t="str">
+        <x:v>Intuit</x:v>
+      </x:c>
+      <x:c r="B11" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="16" t="str">
+        <x:v>H&amp;M</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="16" t="str">
+        <x:v>Unassigned</x:v>
+      </x:c>
+      <x:c r="B13" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="16" t="str">
+        <x:v>Unmapped</x:v>
+      </x:c>
+      <x:c r="B14" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2010,7 +2123,7 @@
         <x:v>Snapshot Date</x:v>
       </x:c>
       <x:c r="B2" s="16" t="str">
-        <x:v>14 Oct 2026</x:v>
+        <x:v>15 Oct 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2018,7 +2131,7 @@
         <x:v>Overall Internal Attrition</x:v>
       </x:c>
       <x:c r="B3" s="18" t="n">
-        <x:v>0.35</x:v>
+        <x:v>0.43</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -2052,36 +2165,6 @@
       <x:c r="B7" s="16" t="str">
         <x:v>No exit-interview data supplied in the current workbook</x:v>
       </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="38" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="100" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="17" t="str">
-        <x:v>Category</x:v>
-      </x:c>
-      <x:c r="B1" s="17" t="str">
-        <x:v>Observation</x:v>
-      </x:c>
-      <x:c r="C1" s="17" t="str">
-        <x:v>Details</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="16" t="str"/>
-      <x:c r="B2" s="16" t="str"/>
-      <x:c r="C2" s="16" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Publish latest Bench workbook snapshot and matching template
</commit_message>
<xml_diff>
--- a/Aditi_Workforce_Dashboard_Upload_Template.xlsx
+++ b/Aditi_Workforce_Dashboard_Upload_Template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active" sheetId="1" r:id="R9d3fa3ff4ea642f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exit" sheetId="2" r:id="R57c0533b52b54c12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions" sheetId="3" r:id="R0d75fb7087a04d8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrition" sheetId="4" r:id="R2c87a8d1e76b475d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active" sheetId="1" r:id="R298c3c2587b84f9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exit" sheetId="2" r:id="R20fcb54403c04cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions" sheetId="3" r:id="R52fd2654fe9843ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrition" sheetId="4" r:id="R058cc92451384869"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -292,6 +292,7 @@
     <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -311,21 +312,24 @@
         <x:v>Department</x:v>
       </x:c>
       <x:c r="F1" s="5" t="str">
+        <x:v>Actual Department</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="str">
         <x:v>Sub Department</x:v>
       </x:c>
-      <x:c r="G1" s="5" t="str">
+      <x:c r="H1" s="5" t="str">
         <x:v>Job Title</x:v>
       </x:c>
-      <x:c r="H1" s="5" t="str">
+      <x:c r="I1" s="5" t="str">
         <x:v>Date Joined</x:v>
       </x:c>
-      <x:c r="I1" s="5" t="str">
+      <x:c r="J1" s="5" t="str">
         <x:v>Client</x:v>
       </x:c>
-      <x:c r="J1" s="5" t="str">
+      <x:c r="K1" s="5" t="str">
         <x:v>Billable</x:v>
       </x:c>
-      <x:c r="K1" s="5" t="str">
+      <x:c r="L1" s="5" t="str">
         <x:v>Category</x:v>
       </x:c>
     </x:row>
@@ -341,6 +345,7 @@
       <x:c r="I2" s="3"/>
       <x:c r="J2" s="3"/>
       <x:c r="K2" s="3"/>
+      <x:c r="L2" s="3"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -394,37 +399,37 @@
         <x:v>Department</x:v>
       </x:c>
       <x:c r="H1" s="5" t="str">
+        <x:v>Actual Department</x:v>
+      </x:c>
+      <x:c r="I1" s="5" t="str">
         <x:v>Sub Department</x:v>
       </x:c>
-      <x:c r="I1" s="5" t="str">
+      <x:c r="J1" s="5" t="str">
         <x:v>Job Title</x:v>
       </x:c>
-      <x:c r="J1" s="5" t="str">
+      <x:c r="K1" s="5" t="str">
         <x:v>Reporting To</x:v>
       </x:c>
-      <x:c r="K1" s="5" t="str">
+      <x:c r="L1" s="5" t="str">
         <x:v>Date Joined</x:v>
       </x:c>
-      <x:c r="L1" s="5" t="str">
+      <x:c r="M1" s="5" t="str">
         <x:v>Exit Date</x:v>
       </x:c>
-      <x:c r="M1" s="5" t="str">
+      <x:c r="N1" s="5" t="str">
         <x:v>Quarter</x:v>
       </x:c>
-      <x:c r="N1" s="5" t="str">
+      <x:c r="O1" s="5" t="str">
         <x:v>Termination Type</x:v>
       </x:c>
-      <x:c r="O1" s="5" t="str">
+      <x:c r="P1" s="5" t="str">
         <x:v>Termination Reason</x:v>
       </x:c>
-      <x:c r="P1" s="5" t="str">
+      <x:c r="Q1" s="5" t="str">
         <x:v>Client </x:v>
       </x:c>
-      <x:c r="Q1" s="5" t="str">
+      <x:c r="R1" s="5" t="str">
         <x:v>Billable</x:v>
-      </x:c>
-      <x:c r="R1" s="5" t="str">
-        <x:v>Category</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -467,751 +472,418 @@
     <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="70" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="70" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="30" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="30" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>ODC positions</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str"/>
-      <x:c r="C1" s="3" t="str"/>
-      <x:c r="D1" s="3" t="str"/>
-      <x:c r="E1" s="3" t="str"/>
-      <x:c r="F1" s="3" t="str"/>
-      <x:c r="G1" s="3" t="str"/>
-      <x:c r="H1" s="3" t="str"/>
-      <x:c r="I1" s="3" t="str"/>
-      <x:c r="J1" s="3" t="str"/>
-      <x:c r="K1" s="3" t="str"/>
-      <x:c r="L1" s="3" t="str"/>
-      <x:c r="M1" s="3" t="str"/>
-      <x:c r="N1" s="3" t="str"/>
-      <x:c r="O1" s="3" t="str"/>
-    </x:row>
-    <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="5" t="str">
-        <x:v>POSITION TYPE</x:v>
-      </x:c>
-      <x:c r="B2" s="5" t="str">
-        <x:v>JOB TITLE</x:v>
-      </x:c>
-      <x:c r="C2" s="5" t="str">
-        <x:v>JOB COMPANY</x:v>
-      </x:c>
-      <x:c r="D2" s="5" t="str">
-        <x:v>JOBDIVA REF NO</x:v>
-      </x:c>
-      <x:c r="E2" s="5" t="str">
-        <x:v>OPTIONAL REF NO</x:v>
-      </x:c>
-      <x:c r="F2" s="5" t="str">
-        <x:v>COUNTRY</x:v>
-      </x:c>
-      <x:c r="G2" s="5" t="str">
-        <x:v>START DATE</x:v>
-      </x:c>
-      <x:c r="H2" s="5" t="str">
-        <x:v>JOB STATUS</x:v>
-      </x:c>
-      <x:c r="I2" s="5" t="str">
-        <x:v>DIVISION NAME</x:v>
-      </x:c>
-      <x:c r="J2" s="5" t="str">
-        <x:v>POSITIONS</x:v>
-      </x:c>
-      <x:c r="K2" s="5" t="str">
-        <x:v>FILLS</x:v>
-      </x:c>
-      <x:c r="L2" s="5" t="str"/>
-      <x:c r="M2" s="5" t="str"/>
-      <x:c r="N2" s="5" t="str"/>
-      <x:c r="O2" s="5" t="str"/>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>BU</x:v>
+      </x:c>
+      <x:c r="B1" s="5" t="str">
+        <x:v>Approved HC</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
+        <x:v>Active HC</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>Serving Notice</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>Open Positions</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>Offered</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="str">
+        <x:v>TBH</x:v>
+      </x:c>
+      <x:c r="H1" s="5" t="str">
+        <x:v>Hold Positions</x:v>
+      </x:c>
+      <x:c r="I1" s="5" t="str">
+        <x:v>Long leave</x:v>
+      </x:c>
+      <x:c r="J1" s="5" t="str">
+        <x:v>PIPs</x:v>
+      </x:c>
+      <x:c r="K1" s="5" t="str">
+        <x:v>Serving Notice </x:v>
+      </x:c>
+      <x:c r="L1" s="5" t="str">
+        <x:v>Bench</x:v>
+      </x:c>
+      <x:c r="M1" s="5" t="str">
+        <x:v>Open Position Remarks</x:v>
+      </x:c>
+      <x:c r="N1" s="5" t="str">
+        <x:v>TBJ (Offered)</x:v>
+      </x:c>
+      <x:c r="O1" s="5" t="str">
+        <x:v>Long Leave</x:v>
+      </x:c>
+      <x:c r="P1" s="5" t="str">
+        <x:v>PIP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="3" t="str">
+        <x:v>US recruited (TOD &amp; DES)</x:v>
+      </x:c>
+      <x:c r="B2" s="3" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="C2" s="3" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="D2" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="3" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F2" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G2" s="3" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H2" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I2" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J2" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K2" s="3" t="str"/>
+      <x:c r="L2" s="3" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="M2" s="3" t="str">
+        <x:v>7 US Technical Recruiter</x:v>
+      </x:c>
+      <x:c r="N2" s="3" t="str"/>
+      <x:c r="O2" s="3" t="str"/>
+      <x:c r="P2" s="3" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>Contract</x:v>
-      </x:c>
-      <x:c r="B3" s="3" t="str">
-        <x:v>Security Software Designer</x:v>
-      </x:c>
-      <x:c r="C3" s="3" t="str">
-        <x:v>Wabtec Corporation</x:v>
-      </x:c>
-      <x:c r="D3" s="3" t="str">
-        <x:v>26-02456</x:v>
-      </x:c>
-      <x:c r="E3" s="3" t="str">
-        <x:v>26-02456</x:v>
-      </x:c>
-      <x:c r="F3" s="3" t="str">
-        <x:v>India</x:v>
+        <x:v>India Recruitment ( TOD &amp; DES)</x:v>
+      </x:c>
+      <x:c r="B3" s="3" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="C3" s="3" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D3" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F3" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G3" s="3" t="n">
-        <x:v>46132</x:v>
-      </x:c>
-      <x:c r="H3" s="3" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
-      <x:c r="I3" s="3" t="str">
-        <x:v>Services</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H3" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I3" s="3" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J3" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K3" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K3" s="3" t="str"/>
       <x:c r="L3" s="3" t="str"/>
-      <x:c r="M3" s="3" t="str"/>
+      <x:c r="M3" s="3" t="str">
+        <x:v>1 Technical Recruiter </x:v>
+      </x:c>
       <x:c r="N3" s="3" t="str"/>
       <x:c r="O3" s="3" t="str"/>
+      <x:c r="P3" s="3" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="3" t="str">
-        <x:v>Contract</x:v>
-      </x:c>
-      <x:c r="B4" s="3" t="str">
-        <x:v>Senior Cybersecurity Engineer</x:v>
-      </x:c>
-      <x:c r="C4" s="3" t="str">
-        <x:v>Wabtec Corporation</x:v>
-      </x:c>
-      <x:c r="D4" s="3" t="str">
-        <x:v>26-03466</x:v>
-      </x:c>
-      <x:c r="E4" s="3" t="str">
-        <x:v>26-03466</x:v>
-      </x:c>
-      <x:c r="F4" s="3" t="str">
-        <x:v>India</x:v>
+        <x:v>Client Services</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C4" s="3" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D4" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G4" s="3" t="n">
-        <x:v>46194</x:v>
-      </x:c>
-      <x:c r="H4" s="3" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
-      <x:c r="I4" s="3" t="str">
-        <x:v>Services</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I4" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J4" s="3" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="K4" s="3" t="n">
-        <x:v>2</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K4" s="3" t="str"/>
       <x:c r="L4" s="3" t="str"/>
-      <x:c r="M4" s="3" t="str"/>
+      <x:c r="M4" s="3" t="str">
+        <x:v>No Open Positions</x:v>
+      </x:c>
       <x:c r="N4" s="3" t="str"/>
       <x:c r="O4" s="3" t="str"/>
+      <x:c r="P4" s="3" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="str">
-        <x:v>Contract</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="str">
-        <x:v>Senior RPG Developer(IBM i / AS400)</x:v>
-      </x:c>
-      <x:c r="C5" s="3" t="str">
-        <x:v>Wabtec Corporation</x:v>
-      </x:c>
-      <x:c r="D5" s="3" t="str">
-        <x:v>26-05532</x:v>
-      </x:c>
-      <x:c r="E5" s="3" t="str">
-        <x:v>26-05532</x:v>
-      </x:c>
-      <x:c r="F5" s="3" t="str">
-        <x:v>India</x:v>
+        <x:v>Business Operations</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="C5" s="3" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="D5" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="3" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F5" s="3" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="3" t="n">
-        <x:v>46272</x:v>
-      </x:c>
-      <x:c r="H5" s="3" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
-      <x:c r="I5" s="3" t="str">
-        <x:v>Services</x:v>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H5" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" s="3" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J5" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K5" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L5" s="3" t="str"/>
-      <x:c r="M5" s="3" t="str"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="3" t="str"/>
+      <x:c r="L5" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M5" s="3" t="str">
+        <x:v>1 Engagement Specialist ,1 HR Service Delivery, 1 Desktop Support Executive, 1 Global Leader – Learning &amp; Talent Development, 2 HRMS Administrator, 1 Business Process / Systems Analyst, 1 Global Employee Engagement Manager, 1 Global Compensation &amp; Total Rewards Manager</x:v>
+      </x:c>
       <x:c r="N5" s="3" t="str"/>
       <x:c r="O5" s="3" t="str"/>
+      <x:c r="P5" s="3" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="3" t="str">
-        <x:v>Contract</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="str">
-        <x:v>Senior Cybersecurity Engineer</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="str">
-        <x:v>Wabtec Corporation</x:v>
-      </x:c>
-      <x:c r="D6" s="3" t="str">
-        <x:v>26-05722</x:v>
-      </x:c>
-      <x:c r="E6" s="3" t="str">
-        <x:v>26-05722</x:v>
-      </x:c>
-      <x:c r="F6" s="3" t="str">
-        <x:v>India</x:v>
+        <x:v>ODC</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C6" s="3" t="n">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="D6" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="3" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F6" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G6" s="3" t="n">
-        <x:v>46279</x:v>
-      </x:c>
-      <x:c r="H6" s="3" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
-      <x:c r="I6" s="3" t="str">
-        <x:v>Services</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H6" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I6" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K6" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K6" s="3" t="str"/>
       <x:c r="L6" s="3" t="str"/>
       <x:c r="M6" s="3" t="str"/>
       <x:c r="N6" s="3" t="str"/>
       <x:c r="O6" s="3" t="str"/>
+      <x:c r="P6" s="3" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="3" t="str">
-        <x:v>Contract</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="str">
-        <x:v>Senior Automation Engineer</x:v>
-      </x:c>
-      <x:c r="C7" s="3" t="str">
-        <x:v>Wabtec Corporation</x:v>
-      </x:c>
-      <x:c r="D7" s="3" t="str">
-        <x:v>26-05723</x:v>
-      </x:c>
-      <x:c r="E7" s="3" t="str">
-        <x:v>26-05723</x:v>
-      </x:c>
-      <x:c r="F7" s="3" t="str">
-        <x:v>India</x:v>
+        <x:v>ODC Internal</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C7" s="3" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D7" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="3" t="n">
-        <x:v>46272</x:v>
-      </x:c>
-      <x:c r="H7" s="3" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
-      <x:c r="I7" s="3" t="str">
-        <x:v>Services</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H7" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J7" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K7" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" s="3" t="str"/>
       <x:c r="L7" s="3" t="str"/>
       <x:c r="M7" s="3" t="str"/>
       <x:c r="N7" s="3" t="str"/>
       <x:c r="O7" s="3" t="str"/>
+      <x:c r="P7" s="3" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="3" t="str">
-        <x:v>Contract</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="str">
-        <x:v>Senior Cybersecurity Engineer</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="str">
-        <x:v>Wabtec Corporation</x:v>
-      </x:c>
-      <x:c r="D8" s="3" t="str">
-        <x:v>26-06391</x:v>
-      </x:c>
-      <x:c r="E8" s="3" t="str">
-        <x:v>26-06391</x:v>
-      </x:c>
-      <x:c r="F8" s="3" t="str">
-        <x:v>India</x:v>
+        <x:v>ODC internal Billable</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="n">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="3" t="n">
-        <x:v>46303</x:v>
-      </x:c>
-      <x:c r="H8" s="3" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
-      <x:c r="I8" s="3" t="str">
-        <x:v>Services</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J8" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K8" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="3" t="str"/>
       <x:c r="L8" s="3" t="str"/>
       <x:c r="M8" s="3" t="str"/>
       <x:c r="N8" s="3" t="str"/>
       <x:c r="O8" s="3" t="str"/>
+      <x:c r="P8" s="3" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="3" t="str">
-        <x:v>Contract</x:v>
-      </x:c>
-      <x:c r="B9" s="3" t="str">
-        <x:v>Production Support Engineer (L2)</x:v>
-      </x:c>
-      <x:c r="C9" s="3" t="str">
-        <x:v>Wabtec Corporation</x:v>
-      </x:c>
-      <x:c r="D9" s="3" t="str">
-        <x:v>26-06425</x:v>
-      </x:c>
-      <x:c r="E9" s="3" t="str">
-        <x:v>26-06425</x:v>
-      </x:c>
-      <x:c r="F9" s="3" t="str">
-        <x:v>India</x:v>
+        <x:v>ODC Fixed Term Contractors</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C9" s="3" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="D9" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="3" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F9" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="3" t="n">
-        <x:v>46306</x:v>
-      </x:c>
-      <x:c r="H9" s="3" t="str">
-        <x:v>OPEN</x:v>
-      </x:c>
-      <x:c r="I9" s="3" t="str">
-        <x:v>Services</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="3" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J9" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K9" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K9" s="3" t="str"/>
       <x:c r="L9" s="3" t="str"/>
-      <x:c r="M9" s="3" t="str"/>
+      <x:c r="M9" s="3" t="str">
+        <x:v>7 positions are billable FTC</x:v>
+      </x:c>
       <x:c r="N9" s="3" t="str"/>
       <x:c r="O9" s="3" t="str"/>
+      <x:c r="P9" s="3" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="3" t="str">
-        <x:v>Corporate </x:v>
-      </x:c>
-      <x:c r="B10" s="3" t="str"/>
-      <x:c r="C10" s="3" t="str"/>
-      <x:c r="D10" s="3" t="str"/>
-      <x:c r="E10" s="3" t="str"/>
-      <x:c r="F10" s="3" t="str"/>
-      <x:c r="G10" s="3" t="str"/>
-      <x:c r="H10" s="3" t="str"/>
-      <x:c r="I10" s="3" t="str"/>
-      <x:c r="J10" s="3" t="str"/>
+        <x:v>Total</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="n">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="n">
+        <x:v>328</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J10" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="K10" s="3" t="str"/>
       <x:c r="L10" s="3" t="str"/>
       <x:c r="M10" s="3" t="str"/>
       <x:c r="N10" s="3" t="str"/>
       <x:c r="O10" s="3" t="str"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="3" t="str">
-        <x:v>BU</x:v>
-      </x:c>
-      <x:c r="B11" s="3" t="str">
-        <x:v>Approved HC</x:v>
-      </x:c>
-      <x:c r="C11" s="3" t="str">
-        <x:v>Active HC</x:v>
-      </x:c>
-      <x:c r="D11" s="3" t="str">
-        <x:v>Serving Notice</x:v>
-      </x:c>
-      <x:c r="E11" s="3" t="str">
-        <x:v>Open Positions</x:v>
-      </x:c>
-      <x:c r="F11" s="3" t="str">
-        <x:v>Offered</x:v>
-      </x:c>
-      <x:c r="G11" s="3" t="str">
-        <x:v>TBH</x:v>
-      </x:c>
-      <x:c r="H11" s="3" t="str">
-        <x:v>Hold Positions</x:v>
-      </x:c>
-      <x:c r="I11" s="3" t="str">
-        <x:v>Long leave</x:v>
-      </x:c>
-      <x:c r="J11" s="3" t="str">
-        <x:v>PIPs</x:v>
-      </x:c>
-      <x:c r="K11" s="3" t="str">
-        <x:v>Serving Notice </x:v>
-      </x:c>
-      <x:c r="L11" s="3" t="str">
-        <x:v>Open Position Remarks</x:v>
-      </x:c>
-      <x:c r="M11" s="3" t="str">
-        <x:v>TBJ (Offered)</x:v>
-      </x:c>
-      <x:c r="N11" s="3" t="str">
-        <x:v>Long Leave</x:v>
-      </x:c>
-      <x:c r="O11" s="3" t="str">
-        <x:v>PIP</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="3" t="str">
-        <x:v>US recruited (TOD &amp; DES)</x:v>
-      </x:c>
-      <x:c r="B12" s="3" t="n">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="C12" s="3" t="n">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="D12" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E12" s="3" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="F12" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G12" s="3" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="H12" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I12" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J12" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K12" s="3" t="str"/>
-      <x:c r="L12" s="3" t="str">
-        <x:v>7 US Technical Recruiter</x:v>
-      </x:c>
-      <x:c r="M12" s="3" t="str"/>
-      <x:c r="N12" s="3" t="str"/>
-      <x:c r="O12" s="3" t="str"/>
-    </x:row>
-    <x:row r="13" ht="34" customHeight="1">
-      <x:c r="A13" s="5" t="str">
-        <x:v>India Recruitment ( TOD &amp; DES)</x:v>
-      </x:c>
-      <x:c r="B13" s="5" t="n">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C13" s="5" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="D13" s="5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E13" s="5" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F13" s="5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G13" s="5" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H13" s="5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I13" s="5" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J13" s="5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K13" s="5" t="str"/>
-      <x:c r="L13" s="5" t="str">
-        <x:v>1 Technical Recruiter </x:v>
-      </x:c>
-      <x:c r="M13" s="5" t="str"/>
-      <x:c r="N13" s="5" t="str"/>
-      <x:c r="O13" s="5" t="str"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="3" t="str">
-        <x:v>Client Services</x:v>
-      </x:c>
-      <x:c r="B14" s="3" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C14" s="3" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="D14" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E14" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F14" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G14" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H14" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I14" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J14" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K14" s="3" t="str"/>
-      <x:c r="L14" s="3" t="str">
-        <x:v>No Open Positions</x:v>
-      </x:c>
-      <x:c r="M14" s="3" t="str"/>
-      <x:c r="N14" s="3" t="str"/>
-      <x:c r="O14" s="3" t="str"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="3" t="str">
-        <x:v>Business Operations</x:v>
-      </x:c>
-      <x:c r="B15" s="3" t="n">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="C15" s="3" t="n">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="D15" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E15" s="3" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F15" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G15" s="3" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H15" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I15" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J15" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K15" s="3" t="str"/>
-      <x:c r="L15" s="3" t="str">
-        <x:v>1 Engagement Specialist ,1 HR Service Delivery, 1 Desktop Support Executive, 1 Global Leader – Learning &amp; Talent Development, 2 HRMS Administrator, 1 Business Process / Systems Analyst, 1 Global Employee Engagement Manager, 1 Global Compensation &amp; Total Rewards Manager, 1 Director – Global HR Service Center</x:v>
-      </x:c>
-      <x:c r="M15" s="3" t="str"/>
-      <x:c r="N15" s="3" t="str"/>
-      <x:c r="O15" s="3" t="str"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="3" t="str">
-        <x:v>ODC</x:v>
-      </x:c>
-      <x:c r="B16" s="3" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C16" s="3" t="n">
-        <x:v>143</x:v>
-      </x:c>
-      <x:c r="D16" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E16" s="3" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="F16" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G16" s="3" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H16" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I16" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J16" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K16" s="3" t="str"/>
-      <x:c r="L16" s="3" t="str"/>
-      <x:c r="M16" s="3" t="str"/>
-      <x:c r="N16" s="3" t="str"/>
-      <x:c r="O16" s="3" t="str"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="3" t="str">
-        <x:v>ODC Internal</x:v>
-      </x:c>
-      <x:c r="B17" s="3" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C17" s="3" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="D17" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E17" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F17" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G17" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H17" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I17" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J17" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K17" s="3" t="str"/>
-      <x:c r="L17" s="3" t="str"/>
-      <x:c r="M17" s="3" t="str"/>
-      <x:c r="N17" s="3" t="str"/>
-      <x:c r="O17" s="3" t="str"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="3" t="str">
-        <x:v>ODC internal Billable</x:v>
-      </x:c>
-      <x:c r="B18" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C18" s="3" t="n">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="D18" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E18" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F18" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G18" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H18" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I18" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J18" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K18" s="3" t="str"/>
-      <x:c r="L18" s="3" t="str"/>
-      <x:c r="M18" s="3" t="str"/>
-      <x:c r="N18" s="3" t="str"/>
-      <x:c r="O18" s="3" t="str"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="3" t="str">
-        <x:v>ODC Fixed Term Contractors</x:v>
-      </x:c>
-      <x:c r="B19" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C19" s="3" t="n">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="D19" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E19" s="3" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="F19" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G19" s="3" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H19" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I19" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J19" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K19" s="3" t="str"/>
-      <x:c r="L19" s="3" t="str">
-        <x:v>9 positions are billable FTC</x:v>
-      </x:c>
-      <x:c r="M19" s="3" t="str"/>
-      <x:c r="N19" s="3" t="str"/>
-      <x:c r="O19" s="3" t="str"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="3" t="str">
-        <x:v>Total</x:v>
-      </x:c>
-      <x:c r="B20" s="3" t="n">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="C20" s="3" t="n">
-        <x:v>451</x:v>
-      </x:c>
-      <x:c r="D20" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E20" s="3" t="n">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="F20" s="3" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G20" s="3" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="H20" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I20" s="3" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J20" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K20" s="3" t="str"/>
-      <x:c r="L20" s="3" t="str"/>
-      <x:c r="M20" s="3" t="str"/>
-      <x:c r="N20" s="3" t="str"/>
-      <x:c r="O20" s="3" t="str"/>
+      <x:c r="P10" s="3" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1370,19 +1042,19 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="S2" s="3" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="T2" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="U2" s="3" t="n">
-        <x:v>56</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="V2" s="6" t="n">
-        <x:v>0.4609053497942387</x:v>
+        <x:v>0.45267489711934156</x:v>
       </x:c>
       <x:c r="W2" s="6" t="n">
-        <x:v>0.5530864197530864</x:v>
+        <x:v>0.5432098765432098</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1427,10 +1099,10 @@
         <x:v>139</x:v>
       </x:c>
       <x:c r="O3" s="3" t="n">
-        <x:v>143</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="P3" s="3" t="n">
-        <x:v>141</x:v>
+        <x:v>142.5</x:v>
       </x:c>
       <x:c r="Q3" s="3" t="n">
         <x:v>8</x:v>
@@ -1448,10 +1120,10 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="V3" s="6" t="n">
-        <x:v>0.19858156028368795</x:v>
+        <x:v>0.19649122807017544</x:v>
       </x:c>
       <x:c r="W3" s="6" t="n">
-        <x:v>0.23829787234042552</x:v>
+        <x:v>0.23578947368421055</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1465,19 +1137,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="D4" s="3" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E4" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F4" s="3" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G4" s="6" t="n">
-        <x:v>0.358974358974359</x:v>
+        <x:v>0.3076923076923077</x:v>
       </x:c>
       <x:c r="H4" s="6" t="n">
-        <x:v>0.43076923076923074</x:v>
+        <x:v>0.36923076923076925</x:v>
       </x:c>
       <x:c r="I4" s="3" t="n">
         <x:v>21</x:v>
@@ -1543,19 +1215,19 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="G5" s="6" t="n">
-        <x:v>0.23225806451612904</x:v>
+        <x:v>0.23376623376623376</x:v>
       </x:c>
       <x:c r="H5" s="6" t="n">
-        <x:v>0.2787096774193548</x:v>
+        <x:v>0.2805194805194805</x:v>
       </x:c>
       <x:c r="I5" s="3" t="n">
         <x:v>79</x:v>
       </x:c>
       <x:c r="J5" s="3" t="n">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="K5" s="3" t="n">
-        <x:v>77.5</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="L5" s="3" t="str"/>
       <x:c r="M5" s="3" t="str">
@@ -1603,28 +1275,28 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="D6" s="3" t="n">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E6" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="3" t="n">
-        <x:v>163</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="G6" s="6" t="n">
-        <x:v>0.5158227848101266</x:v>
+        <x:v>0.525</x:v>
       </x:c>
       <x:c r="H6" s="6" t="n">
-        <x:v>0.6189873417721519</x:v>
+        <x:v>0.6300000000000001</x:v>
       </x:c>
       <x:c r="I6" s="3" t="n">
         <x:v>259</x:v>
       </x:c>
       <x:c r="J6" s="3" t="n">
-        <x:v>373</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="K6" s="3" t="n">
-        <x:v>316</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="L6" s="3" t="str"/>
       <x:c r="M6" s="3" t="str">
@@ -1634,10 +1306,10 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="O6" s="3" t="n">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="P6" s="3" t="n">
-        <x:v>32.5</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="n">
         <x:v>3</x:v>
@@ -1655,10 +1327,10 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="V6" s="6" t="n">
-        <x:v>0.4307692307692308</x:v>
+        <x:v>0.4117647058823529</x:v>
       </x:c>
       <x:c r="W6" s="6" t="n">
-        <x:v>0.5169230769230769</x:v>
+        <x:v>0.49411764705882355</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1681,19 +1353,19 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="G7" s="6" t="n">
-        <x:v>0.19858156028368795</x:v>
+        <x:v>0.19649122807017544</x:v>
       </x:c>
       <x:c r="H7" s="6" t="n">
-        <x:v>0.23829787234042552</x:v>
+        <x:v>0.23578947368421055</x:v>
       </x:c>
       <x:c r="I7" s="3" t="n">
         <x:v>139</x:v>
       </x:c>
       <x:c r="J7" s="3" t="n">
-        <x:v>143</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="K7" s="3" t="n">
-        <x:v>141</x:v>
+        <x:v>142.5</x:v>
       </x:c>
       <x:c r="L7" s="3" t="str"/>
       <x:c r="M7" s="3" t="str">
@@ -1703,10 +1375,10 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="O7" s="3" t="n">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="P7" s="3" t="n">
-        <x:v>77.5</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="n">
         <x:v>4</x:v>
@@ -1724,10 +1396,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="V7" s="6" t="n">
-        <x:v>0.23225806451612904</x:v>
+        <x:v>0.23376623376623376</x:v>
       </x:c>
       <x:c r="W7" s="6" t="n">
-        <x:v>0.2787096774193548</x:v>
+        <x:v>0.2805194805194805</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1772,10 +1444,10 @@
         <x:v>259</x:v>
       </x:c>
       <x:c r="O8" s="3" t="n">
-        <x:v>373</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="P8" s="3" t="n">
-        <x:v>316</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="n">
         <x:v>66</x:v>
@@ -1784,19 +1456,19 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="S8" s="3" t="n">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="T8" s="3" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U8" s="3" t="n">
-        <x:v>163</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="V8" s="6" t="n">
-        <x:v>0.5158227848101266</x:v>
+        <x:v>0.525</x:v>
       </x:c>
       <x:c r="W8" s="6" t="n">
-        <x:v>0.6189873417721519</x:v>
+        <x:v>0.6300000000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1839,23 +1511,23 @@
         <x:v>613</x:v>
       </x:c>
       <x:c r="O9" s="3" t="n">
-        <x:v>699</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="P9" s="3" t="n">
-        <x:v>656</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="str"/>
       <x:c r="R9" s="3" t="str"/>
       <x:c r="S9" s="3" t="str"/>
       <x:c r="T9" s="3" t="str"/>
       <x:c r="U9" s="3" t="n">
-        <x:v>265</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="V9" s="6" t="n">
-        <x:v>0.40396341463414637</x:v>
+        <x:v>0.4069591527987897</x:v>
       </x:c>
       <x:c r="W9" s="6" t="n">
-        <x:v>0.4847560975609756</x:v>
+        <x:v>0.48835098335854765</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1878,19 +1550,19 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="G10" s="6" t="n">
-        <x:v>0.4307692307692308</x:v>
+        <x:v>0.4117647058823529</x:v>
       </x:c>
       <x:c r="H10" s="6" t="n">
-        <x:v>0.5169230769230769</x:v>
+        <x:v>0.49411764705882355</x:v>
       </x:c>
       <x:c r="I10" s="3" t="n">
         <x:v>34</x:v>
       </x:c>
       <x:c r="J10" s="3" t="n">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="K10" s="3" t="n">
-        <x:v>32.5</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="L10" s="3" t="str"/>
       <x:c r="M10" s="3" t="str"/>
@@ -1910,34 +1582,34 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B11" s="3" t="n">
-        <x:v>108</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C11" s="3" t="n">
-        <x:v>78</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="D11" s="3" t="n">
-        <x:v>101</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E11" s="3" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="F11" s="3" t="n">
-        <x:v>265</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="G11" s="6" t="n">
-        <x:v>0.40396341463414637</x:v>
+        <x:v>0.4069591527987897</x:v>
       </x:c>
       <x:c r="H11" s="6" t="n">
-        <x:v>0.4847560975609756</x:v>
+        <x:v>0.48835098335854765</x:v>
       </x:c>
       <x:c r="I11" s="3" t="n">
         <x:v>613</x:v>
       </x:c>
       <x:c r="J11" s="3" t="n">
-        <x:v>699</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="K11" s="3" t="n">
-        <x:v>656</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="L11" s="3" t="str"/>
       <x:c r="M11" s="3" t="str"/>

</xml_diff>